<commit_message>
FlashCard Kaynak dosyası güncellendi
</commit_message>
<xml_diff>
--- a/Uygulamalar ve Kaynakları/APP_Flashcard/Flashcard_Kaynak_Veri.xlsx
+++ b/Uygulamalar ve Kaynakları/APP_Flashcard/Flashcard_Kaynak_Veri.xlsx
@@ -20,12 +20,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t xml:space="preserve">Bilgi edinme değerlendirme kurulu bir itirazı ne kadar sürede karara bağlar?</t>
   </si>
   <si>
     <t xml:space="preserve">30 İş Gününde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilgi edinme kapsamında ilgililer kurul tarafından yapılan itiraza ... gün içinde itiraz ederler.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 gün </t>
   </si>
 </sst>
 </file>
@@ -103,8 +109,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -231,15 +241,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FlashCard Kaynak dosyası güncellendi. 25/07/2026-07.09
</commit_message>
<xml_diff>
--- a/Uygulamalar ve Kaynakları/APP_Flashcard/Flashcard_Kaynak_Veri.xlsx
+++ b/Uygulamalar ve Kaynakları/APP_Flashcard/Flashcard_Kaynak_Veri.xlsx
@@ -1,16 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaan\Desktop\SGK_s-nav_calisma\Uygulamalar ve Kaynakları\APP_Flashcard\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="Sayfa1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
@@ -20,50 +24,32 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t xml:space="preserve">Bilgi edinme değerlendirme kurulu bir itirazı ne kadar sürede karara bağlar?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 İş Gününde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bilgi edinme kapsamında ilgililer kurul tarafından yapılan itiraza ... gün içinde itiraz ederler.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Bilgi edinme değerlendirme kurulu bir itirazı ne kadar sürede karara bağlar?</t>
+  </si>
+  <si>
+    <t>30 İş Gününde</t>
+  </si>
+  <si>
+    <t>Bilgi edinme kapsamında ilgililer kurul tarafından yapılan itiraza ... gün içinde itiraz ederler.</t>
   </si>
   <si>
     <t xml:space="preserve">15 gün </t>
   </si>
+  <si>
+    <t>Görev süresi 10 yıldan az memur kaç gün izin hakkına sahiptir ?</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="162"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="162"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="162"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
       <charset val="162"/>
     </font>
   </fonts>
@@ -76,7 +62,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -84,54 +70,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
@@ -173,14 +136,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -233,18 +196,17 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -252,19 +214,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Sayfa &amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
FlashCard uygulaması 657 SK kaynağı güncellendi ve günlk rapor şablonu dosyasına eklendi
</commit_message>
<xml_diff>
--- a/Uygulamalar ve Kaynakları/APP_Flashcard/Flashcard_Kaynak_Veri.xlsx
+++ b/Uygulamalar ve Kaynakları/APP_Flashcard/Flashcard_Kaynak_Veri.xlsx
@@ -14,6 +14,10 @@
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_ftn1" localSheetId="0">Sayfa1!$A$19</definedName>
+    <definedName name="_ftnref1" localSheetId="0">Sayfa1!$A$16</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -24,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Bilgi edinme değerlendirme kurulu bir itirazı ne kadar sürede karara bağlar?</t>
   </si>
@@ -42,17 +46,237 @@
   </si>
   <si>
     <t>Görev süresi 10 yıldan fazla memur kaç gün izin hakkına sahiptir ?</t>
+  </si>
+  <si>
+    <t>20 gün</t>
+  </si>
+  <si>
+    <t>30 gün</t>
+  </si>
+  <si>
+    <t>Devlet kamu hizmetleri görevlerini ve bu görevlerde çalışan Devlet memurlarını görevlerin gerektirdiği niteliklere ve mesleklere göre sınıflara ayırmaktır.</t>
+  </si>
+  <si>
+    <t>Sınıflandırma</t>
+  </si>
+  <si>
+    <t>Devlet memurlarına, yaptıkları hizmetler için lüzumlu bilgilere ve yetişme şartlarına uygun şekilde, sınıfları içinde en yüksek derecelere kadar ilerleme imkanını sağlamaktır</t>
+  </si>
+  <si>
+    <t>Kariyer</t>
+  </si>
+  <si>
+    <t>Devlet kamu hizmetleri görevlerine girmeyi, sınıflar içinde ilerleme ve yükselmeyi, görevin sona erdirilmesini liyakat sistemine dayandırmak ve bu sistemin eşit imkanlarla uygulanmasında Devlet memurlarını güvenliğe sahip kılmaktır.</t>
+  </si>
+  <si>
+    <t>Liyakat</t>
+  </si>
+  <si>
+    <t>Mevcut kuruluş biçimine bakılmaksızın, Devlet ve diğer kamu tüzel kişiliklerince genel idare esaslarına göre yürütülen asli ve sürekli kamu hizmetlerini ifa ile görevlendirilenler, bu Kanunun uygulanmasında ….. sayılır.</t>
+  </si>
+  <si>
+    <t>memur</t>
+  </si>
+  <si>
+    <t>mali yıl</t>
+  </si>
+  <si>
+    <t>Sözleşmeli personel … sınırlı olarak sözleşme ile çalıştırılmasına karar verilenlerdir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> üç yıllık - otuz gün</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sözleşmeli personel, kapsamda istihdam edilen sözleşmeli personelden aynı kurumda …. çalışma süresini tamamlayanlar bu sürenin bitiminden itibaren …..içinde talepte bulunmaları hâlinde bulundukları yerde aynı unvanlı memur kadrolarına atanır. </t>
+  </si>
+  <si>
+    <t>üç yıl - bir yıl</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sözleşmeli personek can güvenliği ve sağlık sebepleri hariç olmak üzere ….. süreyle başka bir </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>yere atanamaz</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve">. Memur kadrolarına atananlar, aynı yerde en az ….. daha görev yapar. </t>
+    </r>
+  </si>
+  <si>
+    <t>Sözleşmeli personelden memur kadrolarına atananlara iş sonu tazminatı ….</t>
+  </si>
+  <si>
+    <t>ödenmez</t>
+  </si>
+  <si>
+    <r>
+      <t>Sözleşmeli personel seçiminde uygulanacak sınav ile istisnaları, bunlara ödenebilecek ücretlerin üst sınırları ile verilecek iş sonu tazminatı miktarı, kullandırılacak izinler, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>pozisyon unvan ve nitelikleri, (…)</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>14</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> sözleşme fesih halleri, pozisyonların iptali, istihdamına dair hususlar ile sözleşme esas ve usulleri </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t>yurtdışı teşkilatlarında istihdam edilecek personel için ayrıca olmak üzere</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> ..... belirlenir</t>
+    </r>
+  </si>
+  <si>
+    <t>Cumhurbaşkanınca</t>
+  </si>
+  <si>
+    <t>Sözleşmeli personelin görevden uzaklaştırılması ile disipline aykırı fiil ve hâllerin gerçekleşmesi durumunda bu personele verilmesi gereken disiplin cezaları, disiplin cezası vermeye yetkili merciler ve disiplin kurulları ile disipline dair diğer hususlar hakkında Devlet memurlarının tabi olduğu hükümler uygulanır. Ancak, kademe ilerlemesinin durdurulması ve üstü ceza verilmesini gerektiren fiil ve hâllerde disiplin kurulunun kararı alınarak sözleşmeli personelin görevine atamaya ..... onayı ile son verilir.</t>
+  </si>
+  <si>
+    <t>yetkili amirin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devlet memurları bu hususu "Asli Devlet Memurluğuna" atandıktan sonra en geç…. içinde kurumlarınca düzenlenecek merasimle yetkili amirlerin huzurunda yapacakları yeminle belirtirler </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> bir ay</t>
+  </si>
+  <si>
+    <t>Devlet memuru amirinden aldığı emri, Anayasa, kanun, Cumhurbaşkanlığı kararnamesi ve yönetmelik hükümlerine aykırı görürse, ......ve bu aykırılığı o emri verene bildirir. Amir emrinde israr eder ve bu emrini yazı ile yenilerse, memur bu emri yapmağa mecburdur. Ancak emrin yerine getirilmesinden doğacak sorumluluk ..... aittir</t>
+  </si>
+  <si>
+    <t>yerine getirmez  - emri verene</t>
+  </si>
+  <si>
+    <t>Konusu suç teşkil eden emir, hiçbir suretle …..; yerine getiren kimse sorumluluktan kurtulamaz.</t>
+  </si>
+  <si>
+    <t>yerine getirilmez</t>
+  </si>
+  <si>
+    <t>Devlet memurunun kasıt, kusur, ihmal veya tedbirsizliği sonucu idare zarara uğratılmışsa, bu zararın ilgili memur tarafından …... üzerinden ödenmesi esastır.</t>
+  </si>
+  <si>
+    <t>rayiç bedeli</t>
+  </si>
+  <si>
+    <t>Kişiler kamu hukukuna tabi görevlerle ilgili olarak uğradıkları zararlardan dolayı bu görevleri yerine getiren personel aleyhine değil,…. aleyhine dava açarlar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ilgili kurum</t>
+  </si>
+  <si>
+    <t>Devlet dairelerine tevdi veya bu dairelerce tahsil veya muhafaza edilen para ve para hükmündeki değerli kağıtların ilgili personel tarafından zimmete geçirilmesi halinde, zimmete geçirilen miktar, cezai takibat sonucu beklenmeden ..... tarafından hak sahibine ödenir.</t>
+  </si>
+  <si>
+    <t>Hazine</t>
+  </si>
+  <si>
+    <t>Devlet Memurları, kamu görevleri hakkında basına, haber ajanslarına veya radyo ve televizyon kurumlarına bilgi veya demeç veremezler. Bu konuda gerekli bilgi ancak .... yetkili kılacağı görevli illerde ..... veya yetkili kılacağı görevli tarafından verilebilir.</t>
+  </si>
+  <si>
+    <t>bakanın - valiler</t>
+  </si>
+  <si>
+    <t>Devlet memurları hakkındaki ihbar ve şikayetler, garaz veya mücerret hakaret için, uydurma bir suç isnadı suretiyle yapıldığı ve soruşturma veya yargılamanın tabi olduğu kanuni işlem sonucunda bu isnat sabit olmadığı takdirde, merkezde bu memurun ...., illerde .... isnatta bulunanlar hakkında kamu davası açılmasını Cumhuriyet Savcılığından isterler.</t>
+  </si>
+  <si>
+    <t>en büyük amiri - valiler</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="162"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="162"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="162"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="162"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="TR Arial"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="162"/>
     </font>
   </fonts>
@@ -76,9 +300,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -206,44 +445,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15.6"/>
+  <cols>
+    <col min="1" max="1" width="85.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.5546875" style="2"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:2">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:2">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="31.2">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="31.2">
+      <c r="A6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="46.8">
+      <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="46.8">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="46.8">
+      <c r="A10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="31.2">
+      <c r="A11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
+    <row r="12" spans="1:2">
+      <c r="A12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="79.8">
+      <c r="A13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="93.6">
+      <c r="A14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="46.8">
+      <c r="A15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="62.4">
+      <c r="A16" s="3" t="s">
         <v>30</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="31.2">
+      <c r="A17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="31.2">
+      <c r="A18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="31.2">
+      <c r="A19" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="46.8">
+      <c r="A20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="46.8">
+      <c r="A21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="62.4">
+      <c r="A22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Sayfa &amp;P</oddFooter>

</xml_diff>